<commit_message>
Aggiunge 3 nuovi fondi settoriali: Biotech x2 + Cybersecurity
- LU0255977539 Pictet-Biotech-R EUR (Biotecnologia)
- LU1491986011 Pharus Medical Innovation A EUR (Biotecnologia)
- LU2286300988 Allianz Cyber Security AT Cap EUR (Cybersecurity)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1633,8 +1633,6 @@
       <c r="G25" t="n">
         <v>72.4459991455078</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -1825,8 +1823,6 @@
       <c r="G29" t="n">
         <v>12.5559997558594</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -1870,8 +1866,6 @@
       <c r="G30" t="n">
         <v>2717.27099609375</v>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -1964,10 +1958,6 @@
       <c r="G32" t="n">
         <v>21.24</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2001,10 +1991,6 @@
       <c r="G33" t="n">
         <v>184.09</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2038,10 +2024,6 @@
       <c r="G34" t="n">
         <v>155.39</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2075,10 +2057,6 @@
       <c r="G35" t="n">
         <v>8.74</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2112,10 +2090,6 @@
       <c r="G36" t="n">
         <v>100.46</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2149,10 +2123,6 @@
       <c r="G37" t="n">
         <v>220.12</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2186,10 +2156,6 @@
       <c r="G38" t="n">
         <v>16.23</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2223,10 +2189,6 @@
       <c r="G39" t="n">
         <v>2.75</v>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2260,10 +2222,6 @@
       <c r="G40" t="n">
         <v>44.82</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2297,10 +2255,6 @@
       <c r="G41" t="n">
         <v>38.1</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2334,10 +2288,6 @@
       <c r="G42" t="n">
         <v>20.84</v>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2371,10 +2321,6 @@
       <c r="G43" t="n">
         <v>20.74</v>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2408,10 +2354,6 @@
       <c r="G44" t="n">
         <v>22.43</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2445,10 +2387,6 @@
       <c r="G45" t="n">
         <v>1.96</v>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2482,10 +2420,6 @@
       <c r="G46" t="n">
         <v>504.31</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2519,10 +2453,6 @@
       <c r="G47" t="n">
         <v>28.24</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2556,10 +2486,6 @@
       <c r="G48" t="n">
         <v>44.18</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2593,10 +2519,6 @@
       <c r="G49" t="n">
         <v>10.98</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2630,10 +2552,6 @@
       <c r="G50" t="n">
         <v>17.89</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2667,10 +2585,6 @@
       <c r="G51" t="n">
         <v>346.08</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2704,10 +2618,6 @@
       <c r="G52" t="n">
         <v>123.31</v>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2741,10 +2651,6 @@
       <c r="G53" t="n">
         <v>468.6</v>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2778,10 +2684,6 @@
       <c r="G54" t="n">
         <v>289.2</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2815,10 +2717,6 @@
       <c r="G55" t="n">
         <v>269.07</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2852,10 +2750,6 @@
       <c r="G56" t="n">
         <v>257.18</v>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2889,10 +2783,6 @@
       <c r="G57" t="n">
         <v>607.48</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2926,10 +2816,6 @@
       <c r="G58" t="n">
         <v>15.97</v>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2963,10 +2849,6 @@
       <c r="G59" t="n">
         <v>49.36</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3000,10 +2882,6 @@
       <c r="G60" t="n">
         <v>86.75</v>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3037,10 +2915,6 @@
       <c r="G61" t="n">
         <v>23.44</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3074,10 +2948,6 @@
       <c r="G62" t="n">
         <v>15.51</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3111,10 +2981,6 @@
       <c r="G63" t="n">
         <v>484.48</v>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3148,10 +3014,6 @@
       <c r="G64" t="n">
         <v>23.68</v>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3185,10 +3047,6 @@
       <c r="G65" t="n">
         <v>35.67</v>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3222,10 +3080,6 @@
       <c r="G66" t="n">
         <v>9.42</v>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3259,10 +3113,6 @@
       <c r="G67" t="n">
         <v>190.77</v>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3296,10 +3146,6 @@
       <c r="G68" t="n">
         <v>352.45</v>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3333,10 +3179,6 @@
       <c r="G69" t="n">
         <v>43.97</v>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3370,10 +3212,6 @@
       <c r="G70" t="n">
         <v>28.82</v>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3407,10 +3245,6 @@
       <c r="G71" t="n">
         <v>45.2</v>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3444,10 +3278,6 @@
       <c r="G72" t="n">
         <v>27.9</v>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3481,10 +3311,6 @@
       <c r="G73" t="n">
         <v>15.24</v>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3518,10 +3344,6 @@
       <c r="G74" t="n">
         <v>192.08</v>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3555,10 +3377,6 @@
       <c r="G75" t="n">
         <v>12.58</v>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3592,10 +3410,6 @@
       <c r="G76" t="n">
         <v>520.23</v>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3629,10 +3443,6 @@
       <c r="G77" t="n">
         <v>40.79</v>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3666,10 +3476,6 @@
       <c r="G78" t="n">
         <v>160.59</v>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3703,10 +3509,6 @@
       <c r="G79" t="n">
         <v>638.63</v>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3740,10 +3542,6 @@
       <c r="G80" t="n">
         <v>94.66</v>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3777,10 +3575,6 @@
       <c r="G81" t="n">
         <v>185.95</v>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3814,10 +3608,6 @@
       <c r="G82" t="n">
         <v>39.75</v>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3851,10 +3641,6 @@
       <c r="G83" t="n">
         <v>390.27</v>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3888,10 +3674,6 @@
       <c r="G84" t="n">
         <v>214.1</v>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3925,10 +3707,6 @@
       <c r="G85" t="n">
         <v>24.01</v>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3962,10 +3740,6 @@
       <c r="G86" t="n">
         <v>36.74</v>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3999,10 +3773,6 @@
       <c r="G87" t="n">
         <v>370.46</v>
       </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4036,10 +3806,6 @@
       <c r="G88" t="n">
         <v>38.87</v>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4073,10 +3839,6 @@
       <c r="G89" t="n">
         <v>257.59</v>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4110,10 +3872,6 @@
       <c r="G90" t="n">
         <v>14.02</v>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4147,10 +3905,6 @@
       <c r="G91" t="n">
         <v>308.83</v>
       </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4184,10 +3938,6 @@
       <c r="G92" t="n">
         <v>61.39</v>
       </c>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4221,10 +3971,6 @@
       <c r="G93" t="n">
         <v>32.07</v>
       </c>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4258,10 +4004,6 @@
       <c r="G94" t="n">
         <v>20.29</v>
       </c>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4295,10 +4037,6 @@
       <c r="G95" t="n">
         <v>14.81</v>
       </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4332,10 +4070,6 @@
       <c r="G96" t="n">
         <v>202.73</v>
       </c>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4369,10 +4103,96 @@
       <c r="G97" t="n">
         <v>235.43</v>
       </c>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>3</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>LU0255977539</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Pictet-Biotech-R EUR</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Biotecnologia</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>3</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>LU1491986011</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Pharus Medical Innovation A EUR</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Pharus Management</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Biotecnologia</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>3</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>LU2286300988</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Allianz Cyber Security AT Cap EUR</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Allianz Global Investors</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Cybersecurity</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4466,17 +4286,6 @@
           <t>Amundi Funds - Emerging Markets Green Bond G EURO Hedged (C)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4494,16 +4303,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4521,16 +4320,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4548,16 +4337,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4575,16 +4354,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4602,16 +4371,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4629,16 +4388,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4656,16 +4405,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4683,16 +4422,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4710,16 +4439,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4737,16 +4456,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4764,16 +4473,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4791,16 +4490,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4818,16 +4507,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4845,16 +4524,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4872,16 +4541,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4899,16 +4558,6 @@
           <t>Nessun prezzo su FT Markets</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -5001,8 +4650,6 @@
       <c r="G20" t="n">
         <v>1650.0419921875</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5056,8 +4703,6 @@
       <c r="G21" t="n">
         <v>215.658996582031</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5111,8 +4756,6 @@
       <c r="G22" t="n">
         <v>1926.78796386719</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5123,8 +4766,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -5158,8 +4799,6 @@
       <c r="G23" t="n">
         <v>99.568000793457</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5170,8 +4809,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -5221,8 +4858,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -5256,8 +4891,6 @@
       <c r="G25" t="n">
         <v>128.253005981445</v>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5268,8 +4901,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -5319,8 +4950,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -5354,8 +4983,6 @@
       <c r="G27" t="n">
         <v>800.525024414063</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5366,8 +4993,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -5417,8 +5042,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -5452,8 +5075,6 @@
       <c r="G29" t="n">
         <v>1380.40002441406</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5464,8 +5085,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -5499,8 +5118,6 @@
       <c r="G30" t="n">
         <v>1090.80004882813</v>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>HOLD</t>
@@ -5511,8 +5128,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -5562,8 +5177,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -5613,8 +5226,6 @@
           <t>2026-02-26 19:47</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Aggiunge 5 nuovi fondi tematici: Silver Economy, Consumer, Food, Agribusiness
- LU1426102643 Decalia Silver Generation (Silver Economy)
- LU0187079347 Robeco Global Consumer Trends (Consumer Trends)
- LU2211817601 Allianz Food Security (Sicurezza Alimentare)
- LU1805238125 Fidelity Global Consumer Brands (Consumi/Lusso)
- LU0273147594 DWS Global Agribusiness (Agribusiness)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4189,6 +4189,156 @@
         </is>
       </c>
       <c r="F100" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>3</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>LU1426102643</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Decalia Sicav Silver Generation A1 p EUR</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Decalia</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Silver Economy</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>3</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>LU0187079347</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Robeco Global Consumer Trends Eq. D Cap EUR</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Robeco</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Azionari Consumi - Consumer Trends</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>3</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>LU2211817601</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Allianz Food Security AT Cap EUR</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Allianz Global Investors</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Sicurezza Alimentare</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>3</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>LU1805238125</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Fidelity Global Consumer Brands A Cap EUR</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Azionari Consumi/Lusso</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>3</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>LU0273147594</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>DWS Invest Global Agribusiness NC Cap EUR</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>DWS Invest SICAV</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Agribusiness</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
Aggiunge 10 fondi: Acqua, Ambiente, Clima, Risorse Naturali, Metalli
- LU0496367763 Franklin Gold (unhedged)
- LU1951229035 Mirova Thematic Water
- LU1165135440 BNP Paribas Aqua
- IT0005494569 Arca Blue Leaders
- LU0208853274 JPM Natural Resources Acc
- LU0384406244 Vontobel Transition Resources
- LU0503631987 Pictet Global Environmental Opportunities
- LU1914384182 DWS ESG Climate Opportunities
- LU1883319714 Amundi Global Equity Responsible E2
- LU2394008846 JPM Climate Change Solutions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4339,6 +4339,306 @@
         </is>
       </c>
       <c r="F105" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>3</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>LU0496367763</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Franklin Gold and Precious Metals A EUR</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Franklin Templeton</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Metalli Preziosi</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>3</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>LU1951229035</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>NAT Mirova Thematic Water R Cap EUR</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Natixis / Mirova</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Acqua/Ambiente</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>3</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>LU1165135440</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>BNP Paribas Aqua EUR</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>BNP Paribas Funds</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Acqua/Ambiente</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>3</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>IT0005494569</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Arca Blue Leaders</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Arca Fondi SGR</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Blue Economy</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>3</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>LU0208853274</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>JPM Global Natural Resources A Acc EUR</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>JPMorgan Asset Management</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Risorse Naturali</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>3</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>LU0384406244</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Vontobel Transition Resources C EUR</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Vontobel Asset Management</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Transizione Energetica</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>3</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>LU0503631987</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Pictet-Global Environmental Opportunities-R EUR</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Ambiente</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>3</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>LU1914384182</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>DWS Invest ESG Climate Opportunities NC Cap EUR</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>DWS Invest SICAV</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Clima/ESG</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>3</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>LU1883319714</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Amundi F. Global Equity Responsible E2 EUR</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Amundi Asset Management</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Azionari Globali ESG</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>3</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>LU2394008846</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>JPM Climate Change Solutions A Cap EUR</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>JPMorgan Asset Management</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Clima/Energia Pulita</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
Aggiunge 21 fondi: Security/Digital settoriali + 8 monetari + 10 short bond + 1 corporate
Settoriali: Pictet Security (LU0270905242), Pictet Digital (LU0340555134)
Monetari: Fidelity, JPM, Pictet, BGF, Carmignac, Amundi, Candriam, Eurizon
Breve termine: Invesco, Pictet, DPAM, DWS x2, DNCA, Allianz, Amundi, PIMCO, Eurizon
Corporate BT: Euromobiliare

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fondi_monitoraggio.xlsx
+++ b/fondi_monitoraggio.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4639,6 +4639,636 @@
         </is>
       </c>
       <c r="F115" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>3</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>LU0270905242</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Pictet-Security-R EUR</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Sicurezza/Difesa</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>3</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>LU0340555134</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Pictet-Digital-R EUR</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Azionari Settoriali - Digitale</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>3</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>LU0393653836</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Fidelity Euro Cash E Cap EUR</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Fidelity</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>3</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>LU0252499412</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>JPM EUR Money Market VNAV A Acc EUR</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>JPMorgan Asset Management</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>3</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>LU0366536984</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Pictet-Sovereign Short-Term Money Market EUR-R</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>3</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>LU0432366366</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>BGF Euro Reserve C2 Cap EUR</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>BlackRock</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>3</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>FR0010149161</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Carmignac Court Terme A EUR Acc</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Carmignac Gestion</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>3</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>LU0568620990</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Amundi F. Cash EUR F2 EUR</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Amundi Asset Management</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>3</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>LU1434529050</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Candriam Sust. Money Market Euro C EUR</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Candriam</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>3</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>IT0005367773</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Eurizon Tesoreria Euro BM</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Eurizon Capital SGR</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Fondi Monetari</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>3</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>LU0102737730</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Invesco Euro Ultra-Short Term Debt A EUR</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Invesco</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>3</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>LU2009037222</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Pictet-Ultra Short Term Bonds EUR R EUR</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Pictet Asset Management</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>3</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>BE0058191884</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>DPAM B Bonds EUR Short Term 1 Y B Cap EUR</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>DPAM</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>3</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>LU0236145453</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>DWS Invest Short Duration Credit LC Cap EUR</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>DWS Invest SICAV</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>3</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>LU1490785505</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>DNCA Invest Serenite Plus B Cap EUR</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>DNCA Investments</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>3</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>LU1504571149</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Allianz Adv. Fix. Inc. Short Dur. AT Cap EUR</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Allianz Global Investors</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>3</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>LU1499628912</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Amundi S.F. Diversified Short-Term Bond E EUR</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Amundi Asset Management</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>3</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>IE00B90VC092</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PIMCO European Short-Term Opportunities E EUR</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>PIMCO</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>3</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>LU0145656475</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>DWS Invest ESG Euro Bonds Short LD Dis EUR</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>DWS Invest SICAV</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>3</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>IT0000386646</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Eurizon Obbligazioni Euro Breve Termine D Dis</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Eurizon Capital SGR</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Obbligazionari Breve Termine</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>3</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>IT0000380649</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Euromobiliare Euro Short Term Corporate Bond A</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Euromobiliare</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Obbligazionari Corporate</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>